<commit_message>
Fixed some typos in IPO mappings
</commit_message>
<xml_diff>
--- a/ipo_translation/IPO_schemas.xlsx
+++ b/ipo_translation/IPO_schemas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jmccombs/projects/RDS/ccdi/ccdi-api/ipo_translation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED67DDEB-1BD5-D442-9666-32FCDA392BCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCF587CF-5A2E-5B4F-A1CD-9F158BEFA7BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="64000" windowHeight="26380" xr2:uid="{30C529F3-6AAD-4F4A-B2DD-170CB4F69519}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{30C529F3-6AAD-4F4A-B2DD-170CB4F69519}"/>
   </bookViews>
   <sheets>
     <sheet name="subjects.csv" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="109">
   <si>
     <t>Column</t>
   </si>
@@ -289,9 +289,6 @@
     <t>Participant -&gt; Participant, Patient Derived Xenograft -&gt; Patient Derived Xenograft, Cell Line -&gt; Cell Line, Organoid -&gt; Organoid</t>
   </si>
   <si>
-    <t>Male -&gt; M, Female -&gt; F, Unknown -&gt; U, Unspecified -&gt; U, UNDIFFERENTIATED -&gt; UNDIFFERENTIATED</t>
-  </si>
-  <si>
     <t>Unknown, Black or African American, White, Unknown; White, Not allowed to collect, Native Hawaiian or other Pacific Islander, Not Reported, American Indian or Alaska Native, Asian</t>
   </si>
   <si>
@@ -328,9 +325,6 @@
     <t>AMPLICON, ATAC-Seq, Bisulfite-Seq, ChIA-PET, ChIP-Seq, CLONE, CLONEEND, CTS, DNA-Seq, DNase-Hypersensitivity, EST, FAIRE-seq, FINISHING, FL-cDNA, Hi-C, MBD-Seq, MeDIP-Seq, miRNA-Seq, MNase-Seq, MRE-Seq, ncRNA-Seq, Other, POOLCLONE, RAD-Seq, RIP-Seq, RNA-Seq, SELEX, snATAC-Seq, ssRNA-seq, Synthetic-Long-Read, Targeted-Capture, Tethered Chromatin Conformation Capture, Tn-Seq, WCS, WGA, WGS, WXS</t>
   </si>
   <si>
-    <t>AMPLICON -&gt; AMPLICON, ATAC-Seq -&gt; ATAC-Seq, Bisulfite-Seq -&gt; Bisulfite-Seq, ChIA-PET -&gt; ChIA-PET, ChIP-Seq -&gt; ChIP-Seq, CLONE -&gt; CLONE, CLONEEND -&gt; CLONEEND, CTS -&gt; CTS, DNA-Seq -&gt; DNA-Seq, DNase-Hypersensitivity -&gt; DNase-Hypersensitivity, EST -&gt; EST, FAIRE-seq -&gt; FAIRE-seq, FINISHING -&gt; FINISHING, FL-cDNA -&gt; FL-cDNA, Hi-C -&gt; Hi-C, MBD-Seq -&gt; MBD-Seq, MeDIP-Seq -&gt; MeDIP-Seq, miRNA-Seq -&gt; miRNA-Seq, MNase-Seq -&gt; MNase-Seq, MRE-Seq -&gt; MRE-Seq, ncRNA-Seq -&gt; ncRNA-Seq, Other -&gt; Other, POOLCLONE -&gt; POOLCLONE, RAD-Seq -&gt; RAD-Seq, RIP-Seq -&gt; RIP-Seq, RNA-Seq -&gt; RNA-Seq, SELEX -&gt; SELEX, snATAC-Seq -&gt; nsATAC-Seq, ssRNA-seq -&gt; ssRNA-seq, Synthetic-Long-Read -&gt; Synthetic-Long-Read, Targeted-Capture -&gt; Targeted Capture, Tethered Chromatin Conformation Capture -&gt; Tethered Chromatin Conformation Capture, Tn-Seq -&gt; Tn-Seq, WCS -&gt; WCS, WGA -&gt; WGA, WGS -&gt; WGS, WXS -&gt; WXS</t>
-  </si>
-  <si>
     <t>Bulk Cells, Bulk Nuclei, Bulk Tissue, Single-cells, Single-nuclei, Not Reported</t>
   </si>
   <si>
@@ -356,6 +350,21 @@
   </si>
   <si>
     <t>Unknown -&gt; Unknown, U -&gt; Unknown, Black or African American -&gt; Black or African American, White -&gt; White, Not allowed to collect -&gt; Not allowed to collect, Native Hawaiian or other Pacific Islander -&gt; Native Hawaiian or other Pacific Islander, Not Reported -&gt; Not Reported, American Indian or Alaska Native -&gt; American Indian or Alaska Native, Asian -&gt; Asian</t>
+  </si>
+  <si>
+    <t>Male -&gt; M, Female -&gt; F, Unknown -&gt; U, U -&gt; U, Unspecified -&gt; U, UNDIFFERENTIATED -&gt; UNDIFFERENTIATED</t>
+  </si>
+  <si>
+    <t>Real</t>
+  </si>
+  <si>
+    <t>Some IPO inputs are semicolon-separated lists of race values.  Which value should be selected.  Code currently selects the first value.</t>
+  </si>
+  <si>
+    <t>NA' is not supported in the CCDI data model.  Should we replace with zero?</t>
+  </si>
+  <si>
+    <t>AMPLICON -&gt; AMPLICON, ATAC-Seq -&gt; ATAC-Seq, Bisulfite-Seq -&gt; Bisulfite-Seq, ChIA-PET -&gt; ChIA-PET, ChIP-Seq -&gt; ChIP-Seq, CLONE -&gt; CLONE, CLONEEND -&gt; CLONEEND, CTS -&gt; CTS, DNA-Seq -&gt; DNA-Seq, DNase-Hypersensitivity -&gt; DNase-Hypersensitivity, EST -&gt; EST, FAIRE-seq -&gt; FAIRE-seq, FINISHING -&gt; FINISHING, FL-cDNA -&gt; FL-cDNA, Hi-C -&gt; Hi-C, MBD-Seq -&gt; MBD-Seq, MeDIP-Seq -&gt; MeDIP-Seq, miRNA-Seq -&gt; miRNA-Seq, MNase-Seq -&gt; MNase-Seq, MRE-Seq -&gt; MRE-Seq, ncRNA-Seq -&gt; ncRNA-Seq, Other -&gt; Other, POOLCLONE -&gt; POOLCLONE, RAD-Seq -&gt; RAD-Seq, RIP-Seq -&gt; RIP-Seq, RNA-Seq -&gt; RNA-Seq, SELEX -&gt; SELEX, snATAC-Seq -&gt; snATAC-Seq, ssRNA-seq -&gt; ssRNA-seq, Synthetic-Long-Read -&gt; Synthetic-Long-Read, Targeted-Capture -&gt; Targeted Capture, Tethered Chromatin Conformation Capture -&gt; Tethered Chromatin Conformation Capture, Tn-Seq -&gt; Tn-Seq, WCS -&gt; WCS, WGA -&gt; WGA, WGS -&gt; WGS, WXS -&gt; WXS</t>
   </si>
 </sst>
 </file>
@@ -391,9 +400,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -853,13 +863,13 @@
         <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E6" t="s">
         <v>7</v>
       </c>
       <c r="F6" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -873,13 +883,16 @@
         <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>
       </c>
       <c r="F7" t="s">
-        <v>105</v>
+        <v>103</v>
+      </c>
+      <c r="G7" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -893,13 +906,13 @@
         <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E8" t="s">
         <v>9</v>
       </c>
       <c r="F8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -919,7 +932,7 @@
         <v>10</v>
       </c>
       <c r="F9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -927,19 +940,22 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
         <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E10" t="s">
         <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>88</v>
+        <v>87</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -972,9 +988,10 @@
   <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="67.6640625" customWidth="1"/>
+    <col min="2" max="2" width="0.1640625" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="45.1640625" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="255.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="29.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1133,13 +1150,13 @@
         <v>53</v>
       </c>
       <c r="D8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E8" t="s">
         <v>37</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -1153,13 +1170,13 @@
         <v>54</v>
       </c>
       <c r="D9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E9" t="s">
         <v>38</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -1173,13 +1190,13 @@
         <v>55</v>
       </c>
       <c r="D10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E10" t="s">
         <v>39</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -1213,13 +1230,13 @@
         <v>57</v>
       </c>
       <c r="D12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E12" t="s">
         <v>41</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1233,13 +1250,13 @@
         <v>58</v>
       </c>
       <c r="D13" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E13" t="s">
         <v>42</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1253,13 +1270,13 @@
         <v>59</v>
       </c>
       <c r="D14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E14" t="s">
         <v>43</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -1287,7 +1304,7 @@
         <v>45</v>
       </c>
       <c r="B16" t="s">
-        <v>14</v>
+        <v>105</v>
       </c>
       <c r="C16" t="s">
         <v>61</v>
@@ -1307,7 +1324,7 @@
         <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>105</v>
       </c>
       <c r="C17" t="s">
         <v>62</v>
@@ -1493,13 +1510,13 @@
         <v>77</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E8" t="s">
         <v>67</v>
       </c>
       <c r="F8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Fixed misspelling of Tissue in spreadsheet
</commit_message>
<xml_diff>
--- a/ipo_translation/IPO_schemas.xlsx
+++ b/ipo_translation/IPO_schemas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jmccombs/projects/RDS/ccdi/ccdi-api/ipo_translation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCF587CF-5A2E-5B4F-A1CD-9F158BEFA7BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998FA9C7-ECC5-F645-AE00-46E22BD0B0BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{30C529F3-6AAD-4F4A-B2DD-170CB4F69519}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="64000" windowHeight="26380" activeTab="1" xr2:uid="{30C529F3-6AAD-4F4A-B2DD-170CB4F69519}"/>
   </bookViews>
   <sheets>
     <sheet name="subjects.csv" sheetId="1" r:id="rId1"/>
@@ -328,9 +328,6 @@
     <t>Bulk Cells, Bulk Nuclei, Bulk Tissue, Single-cells, Single-nuclei, Not Reported</t>
   </si>
   <si>
-    <t>Bulk Cells -&gt; Bulk Cells, Bulk Nuclei -&gt; Bulk Nuclei, Bulk Tissue -&gt; Bulk Tissiue, Single-cells -&gt; Single-cells, Single-nuclei -&gt; Single-nuclei, Not Reported -&gt; Not Reported</t>
-  </si>
-  <si>
     <t>-80 degrees C, Cryopreserved, EDTA, FFPE, Formalin Fixed - Buffered, Formalin Fixed - Unbuffered, Fresh, Fresh Dissociated, Fresh Dissociated and Single Cell Sorted, Fresh Dissociated and Single Cell Sorted into Plates, Frozen, Liquid Nitrogen, Not Reported, OCT, Snap Frozen, Unknown</t>
   </si>
   <si>
@@ -365,6 +362,9 @@
   </si>
   <si>
     <t>AMPLICON -&gt; AMPLICON, ATAC-Seq -&gt; ATAC-Seq, Bisulfite-Seq -&gt; Bisulfite-Seq, ChIA-PET -&gt; ChIA-PET, ChIP-Seq -&gt; ChIP-Seq, CLONE -&gt; CLONE, CLONEEND -&gt; CLONEEND, CTS -&gt; CTS, DNA-Seq -&gt; DNA-Seq, DNase-Hypersensitivity -&gt; DNase-Hypersensitivity, EST -&gt; EST, FAIRE-seq -&gt; FAIRE-seq, FINISHING -&gt; FINISHING, FL-cDNA -&gt; FL-cDNA, Hi-C -&gt; Hi-C, MBD-Seq -&gt; MBD-Seq, MeDIP-Seq -&gt; MeDIP-Seq, miRNA-Seq -&gt; miRNA-Seq, MNase-Seq -&gt; MNase-Seq, MRE-Seq -&gt; MRE-Seq, ncRNA-Seq -&gt; ncRNA-Seq, Other -&gt; Other, POOLCLONE -&gt; POOLCLONE, RAD-Seq -&gt; RAD-Seq, RIP-Seq -&gt; RIP-Seq, RNA-Seq -&gt; RNA-Seq, SELEX -&gt; SELEX, snATAC-Seq -&gt; snATAC-Seq, ssRNA-seq -&gt; ssRNA-seq, Synthetic-Long-Read -&gt; Synthetic-Long-Read, Targeted-Capture -&gt; Targeted Capture, Tethered Chromatin Conformation Capture -&gt; Tethered Chromatin Conformation Capture, Tn-Seq -&gt; Tn-Seq, WCS -&gt; WCS, WGA -&gt; WGA, WGS -&gt; WGS, WXS -&gt; WXS</t>
+  </si>
+  <si>
+    <t>Bulk Cells -&gt; Bulk Cells, Bulk Nuclei -&gt; Bulk Nuclei, Bulk Tissue -&gt; Bulk Tissue, Single-cells -&gt; Single-cells, Single-nuclei -&gt; Single-nuclei, Not Reported -&gt; Not Reported</t>
   </si>
 </sst>
 </file>
@@ -863,13 +863,13 @@
         <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E6" t="s">
         <v>7</v>
       </c>
       <c r="F6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -889,10 +889,10 @@
         <v>8</v>
       </c>
       <c r="F7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -940,13 +940,13 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C10" t="s">
         <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E10" t="s">
         <v>11</v>
@@ -955,7 +955,7 @@
         <v>87</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -991,7 +991,7 @@
     <col min="1" max="1" width="67.6640625" customWidth="1"/>
     <col min="2" max="2" width="0.1640625" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="45.1640625" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="255.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="72.83203125" customWidth="1"/>
     <col min="5" max="5" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="29.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1236,7 +1236,7 @@
         <v>41</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1256,7 +1256,7 @@
         <v>42</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1270,13 +1270,13 @@
         <v>59</v>
       </c>
       <c r="D14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E14" t="s">
         <v>43</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -1304,7 +1304,7 @@
         <v>45</v>
       </c>
       <c r="B16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C16" t="s">
         <v>61</v>
@@ -1324,7 +1324,7 @@
         <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C17" t="s">
         <v>62</v>
@@ -1510,13 +1510,13 @@
         <v>77</v>
       </c>
       <c r="D8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E8" t="s">
         <v>67</v>
       </c>
       <c r="F8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>